<commit_message>
Add central database configuration button and update CSV files with new entries
</commit_message>
<xml_diff>
--- a/hasil/rekap_error_gui.xlsx
+++ b/hasil/rekap_error_gui.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G592"/>
+  <dimension ref="A1:G602"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22368,6 +22368,379 @@
         </is>
       </c>
     </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>e7e2f6e3-3213-49ee-9112-43604a001373</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>MAJU LANCAR CV</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>DB:data_split_usaha_20261016</t>
+        </is>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>1114</t>
+        </is>
+      </c>
+      <c r="E593" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="F593" t="inlineStr">
+        <is>
+          <t>Page.wait_for_function: Timeout 30000ms exceeded.</t>
+        </is>
+      </c>
+      <c r="G593" t="inlineStr">
+        <is>
+          <t>2026-10-23 03:58:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>7f5ae8d2-ec21-498c-9728-5db99d9e325d</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>AYAM UNGKEP KELILING DIAN LESMANA</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>DB:data_split_usaha_20261016</t>
+        </is>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>1138</t>
+        </is>
+      </c>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="F594" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Locator.wait_for: Timeout 30000ms exceeded.
+Call log:
+  - waiting for locator("div.fasih-form-sidebar &gt; div[title=\"SE2026 - L BLOK II\"]:visible, div.fasih-form-sidebar &gt; div[title=\"BLOK I\"]:visible, div.fasih-form-sidebar &gt; div[title=\"BLOK II\"]:visible").first to be visible
+</t>
+        </is>
+      </c>
+      <c r="G594" t="inlineStr">
+        <is>
+          <t>2026-10-23 04:32:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>f4b288f3-49c9-4144-8539-e4123095d7e2</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>AYAM GEPREK BANG MALIK</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>DB:data_split_usaha_20261016</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>1318</t>
+        </is>
+      </c>
+      <c r="E595" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="F595" t="inlineStr">
+        <is>
+          <t>Tahun operasi '2026' tidak didukung; isian bulanan perlu penanganan manual.</t>
+        </is>
+      </c>
+      <c r="G595" t="inlineStr">
+        <is>
+          <t>2026-10-23 04:49:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>bb04a5b7-c1dd-4749-ad83-bb3785a7f036</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>BU AISYAH</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>DB:data_split_usaha_20261016</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>1323</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="F596" t="inlineStr">
+        <is>
+          <t>Tahun operasi '2026' tidak didukung; isian bulanan perlu penanganan manual.</t>
+        </is>
+      </c>
+      <c r="G596" t="inlineStr">
+        <is>
+          <t>2026-10-23 04:49:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>c656d2be-dd94-47e9-9ce6-9dfa99e0bfda</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>MENJUAL AYAM POTONG(HASANUDIN)</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>DB:data_split_usaha_20261016</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>1328</t>
+        </is>
+      </c>
+      <c r="E597" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="F597" t="inlineStr">
+        <is>
+          <t>Tahun operasi '2026' tidak didukung; isian bulanan perlu penanganan manual.</t>
+        </is>
+      </c>
+      <c r="G597" t="inlineStr">
+        <is>
+          <t>2026-10-23 04:49:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>3eb7a7c4-b61f-4838-bf25-c6f063b8147b</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>USAHA AYAM POTONG AMIRUDIN</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>DB:data_split_usaha_20261016</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>1333</t>
+        </is>
+      </c>
+      <c r="E598" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="F598" t="inlineStr">
+        <is>
+          <t>Tahun operasi '2026' tidak didukung; isian bulanan perlu penanganan manual.</t>
+        </is>
+      </c>
+      <c r="G598" t="inlineStr">
+        <is>
+          <t>2026-10-23 04:49:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>d53f3e48-e396-4417-979b-1aed0a339447</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>INTI YUDA SAMUDRA</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>DB:data_split_usaha_20261016</t>
+        </is>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>1363</t>
+        </is>
+      </c>
+      <c r="E599" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="F599" t="inlineStr">
+        <is>
+          <t>Page.wait_for_function: Timeout 30000ms exceeded.</t>
+        </is>
+      </c>
+      <c r="G599" t="inlineStr">
+        <is>
+          <t>2026-10-23 04:53:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>bf7d9eba-bdae-402b-ae06-fefdafeffc0d</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>SURI NUSANTARA JAYA, PT</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>DB:data_split_usaha_20261016</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>1368</t>
+        </is>
+      </c>
+      <c r="E600" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="F600" t="inlineStr">
+        <is>
+          <t>Tahun operasi '2026' tidak didukung; isian bulanan perlu penanganan manual.</t>
+        </is>
+      </c>
+      <c r="G600" t="inlineStr">
+        <is>
+          <t>2026-10-23 04:54:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>53c8c63e-6605-4f74-a25d-c54bdfbe7e52</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>PERIKANAN</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>DB:data_split_usaha_20261016</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>1398</t>
+        </is>
+      </c>
+      <c r="E601" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="F601" t="inlineStr">
+        <is>
+          <t>Tahun operasi '2026' tidak didukung; isian bulanan perlu penanganan manual.</t>
+        </is>
+      </c>
+      <c r="G601" t="inlineStr">
+        <is>
+          <t>2026-10-23 04:55:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>b0cd5cfa-24cb-4967-ae0d-fc876bf13472</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>NESTARA TELUR (FAUZAN)</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>DB:data_split_usaha_20261016</t>
+        </is>
+      </c>
+      <c r="D602" t="inlineStr">
+        <is>
+          <t>1493</t>
+        </is>
+      </c>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="F602" t="inlineStr">
+        <is>
+          <t>Tahun operasi '2026' tidak didukung; isian bulanan perlu penanganan manual.</t>
+        </is>
+      </c>
+      <c r="G602" t="inlineStr">
+        <is>
+          <t>2026-10-23 05:01:20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add unit tests for preview_fetch_limit function and update database schema
- Introduced a new test case to validate the behavior of the preview_fetch_limit function, ensuring it returns the correct row limits based on input values.
- Added assertions to check for expected outputs and raise ValueError for invalid inputs.
- Updated the status_gui.sqlite3 database file to reflect recent changes.
</commit_message>
<xml_diff>
--- a/hasil/rekap_error_gui.xlsx
+++ b/hasil/rekap_error_gui.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G602"/>
+  <dimension ref="A1:G609"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22741,6 +22741,265 @@
         </is>
       </c>
     </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>161c2b74-1a43-44e7-8cae-f756f0895424</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>JUAL AYAM POTONG SAYUTI</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>DB:data_split_usaha_20261016</t>
+        </is>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>1326</t>
+        </is>
+      </c>
+      <c r="E603" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="F603" t="inlineStr">
+        <is>
+          <t>Tahun operasi '2026' tidak didukung; isian bulanan perlu penanganan manual.</t>
+        </is>
+      </c>
+      <c r="G603" t="inlineStr">
+        <is>
+          <t>2026-10-23 11:39:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>867dc247-6a0d-4e7f-8aad-20c424569e29</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>FROZEN FOOD (TRI JOKO PURNOMO)</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>DB:data_split_usaha_20261016</t>
+        </is>
+      </c>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>1551</t>
+        </is>
+      </c>
+      <c r="E604" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="F604" t="inlineStr">
+        <is>
+          <t>Tahun operasi '2026' tidak didukung; isian bulanan perlu penanganan manual.</t>
+        </is>
+      </c>
+      <c r="G604" t="inlineStr">
+        <is>
+          <t>2026-10-23 11:43:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>dffa3315-1549-4056-9c62-a532d9b29376</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>TOKO AL-GHIFARI</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>DB:data_split_usaha_20261016</t>
+        </is>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>1851</t>
+        </is>
+      </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="F605" t="inlineStr">
+        <is>
+          <t>Tahun operasi '2026' tidak didukung; isian bulanan perlu penanganan manual.</t>
+        </is>
+      </c>
+      <c r="G605" t="inlineStr">
+        <is>
+          <t>2026-10-23 11:46:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>77388f5e-05d2-4e44-9ed0-bf49eb802eed</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>DD AUTO MOBILINDO</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>DB:data_split_usaha_20261016</t>
+        </is>
+      </c>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>1901</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="F606" t="inlineStr">
+        <is>
+          <t>Tahun operasi '2026' tidak didukung; isian bulanan perlu penanganan manual.</t>
+        </is>
+      </c>
+      <c r="G606" t="inlineStr">
+        <is>
+          <t>2026-10-23 11:46:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>a8176203-88ea-4acb-a97e-b9a9effe5657</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TOKO BAHAN BANGUNAN </t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>DB:data_split_usaha_20261016</t>
+        </is>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>2926</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="F607" t="inlineStr">
+        <is>
+          <t>Tahun operasi '2026' tidak didukung; isian bulanan perlu penanganan manual.</t>
+        </is>
+      </c>
+      <c r="G607" t="inlineStr">
+        <is>
+          <t>2026-10-23 11:57:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>1d78c670-0f4d-403f-adb2-7b96c16e5aa3</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>CUCI PLASTIK (MAIN)</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>DB:data_split_usaha_20261016</t>
+        </is>
+      </c>
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>3676</t>
+        </is>
+      </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="F608" t="inlineStr">
+        <is>
+          <t>Tahun operasi '2026' tidak didukung; isian bulanan perlu penanganan manual.</t>
+        </is>
+      </c>
+      <c r="G608" t="inlineStr">
+        <is>
+          <t>2026-10-23 12:06:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>a02a532b-4498-458a-820d-77eb36372e27</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>SORTIR RONGSOKAN (SAEFUL)</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>DB:data_split_usaha_20261016</t>
+        </is>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>3701</t>
+        </is>
+      </c>
+      <c r="E609" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="F609" t="inlineStr">
+        <is>
+          <t>Tahun operasi '2026' tidak didukung; isian bulanan perlu penanganan manual.</t>
+        </is>
+      </c>
+      <c r="G609" t="inlineStr">
+        <is>
+          <t>2026-10-23 12:06:26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>